<commit_message>
TID Tanda 1: quitar 5 contactos internacionales (USA) - solo Mexico
</commit_message>
<xml_diff>
--- a/GrowProkure/04-GoToMarket/TID_Tanda1_contactos.xlsx
+++ b/GrowProkure/04-GoToMarket/TID_Tanda1_contactos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I131"/>
+  <dimension ref="A1:I126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -504,7 +504,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -537,13 +536,11 @@
           <t>Estado de Mexico</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -576,13 +573,11 @@
           <t>Aguascalientes</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -615,13 +610,11 @@
           <t>Puebla</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -654,13 +647,11 @@
           <t>CDMX</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -693,13 +684,11 @@
           <t>Estado de Mexico</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -742,7 +731,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -785,7 +773,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -828,7 +815,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -871,7 +857,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -914,7 +899,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -957,7 +941,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1000,7 +983,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1043,7 +1025,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1133,7 +1114,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1171,7 +1151,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1214,7 +1193,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1257,7 +1235,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1300,7 +1277,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1338,7 +1314,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1381,7 +1356,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1424,7 +1398,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1452,13 +1425,11 @@
           <t>sergio.castillo@apsolutions.com.mx</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1491,13 +1462,11 @@
           <t>Nuevo Leon</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1530,13 +1499,11 @@
           <t>Tamaulipas</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1569,13 +1536,11 @@
           <t>Baja California</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1603,13 +1568,11 @@
           <t>cesar_blas@baxter.com</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1642,13 +1605,11 @@
           <t>Tlaxcala</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1681,13 +1642,11 @@
           <t>Estado de Mexico</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1720,7 +1679,6 @@
           <t>San Luis Potosi</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>MX</t>
@@ -1763,13 +1721,11 @@
           <t>Nuevo Leon</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1802,13 +1758,11 @@
           <t>Nuevo Leon</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1841,13 +1795,11 @@
           <t>Chihuahua</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1875,13 +1827,11 @@
           <t>enava@dixon.com.mx</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1914,13 +1864,11 @@
           <t>Chihuahua</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1953,13 +1901,11 @@
           <t>Chihuahua</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1992,13 +1938,11 @@
           <t>Chihuahua</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
       <c r="H39" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2031,13 +1975,11 @@
           <t>Jalisco</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
       <c r="H40" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2070,13 +2012,11 @@
           <t>Jalisco</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
       <c r="H41" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2109,13 +2049,11 @@
           <t>Estado de Mexico</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
       <c r="H42" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2148,13 +2086,11 @@
           <t>Tamaulipas</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2187,13 +2123,11 @@
           <t>Tamaulipas</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
       <c r="H44" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2221,13 +2155,11 @@
           <t>tania.olive@honeywell.com</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2260,13 +2192,11 @@
           <t>Nuevo Leon</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2299,13 +2229,11 @@
           <t>Nuevo Leon</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2338,13 +2266,11 @@
           <t>Chihuahua</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
       <c r="H48" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2377,13 +2303,11 @@
           <t>Nuevo Leon</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr"/>
       <c r="H49" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2411,13 +2335,11 @@
           <t>compras@vlar.mx</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
       <c r="H50" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2450,13 +2372,11 @@
           <t>Estado de Mexico</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2484,13 +2404,11 @@
           <t>mario.hughes@jci.com</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2523,13 +2441,11 @@
           <t>Nuevo Leon</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2539,36 +2455,34 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Key Plastics</t>
+          <t>LEGO Group</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>D. Spiteri</t>
+          <t>Luis Castro</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Compras/Contacto</t>
+          <t>NPI &amp; Pad Printing Senior Engineer</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>dspiteri@keyplastics.com</t>
+          <t>luis.castro@lego.com</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr"/>
+          <t>Nuevo Leon</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2578,36 +2492,34 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>LEGO Group</t>
+          <t>La Cazadora</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Luis Castro</t>
+          <t>Lupita Garduno</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>NPI &amp; Pad Printing Senior Engineer</t>
+          <t>Compras/Contacto</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>luis.castro@lego.com</t>
+          <t>lupita.garduno@lacazadora.com.mx</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Nuevo Leon</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr"/>
+          <t>Estado de Mexico</t>
+        </is>
+      </c>
       <c r="H55" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2617,36 +2529,34 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>La Cazadora</t>
+          <t>Mutsutech</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Lupita Garduno</t>
+          <t>Jorge Gonzalez</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Compras/Contacto</t>
+          <t>CS Department Manager</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>lupita.garduno@lacazadora.com.mx</t>
+          <t>lgonzalez@mutsutech.com.mx</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Estado de Mexico</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr"/>
+          <t>Nuevo Leon</t>
+        </is>
+      </c>
       <c r="H56" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2656,36 +2566,34 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Mutsutech</t>
+          <t>Nattura Laboratorios</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Jorge Gonzalez</t>
+          <t>Aurora Becerra</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>CS Department Manager</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>lgonzalez@mutsutech.com.mx</t>
+          <t>aurora.becerra@natturalabs.com</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Nuevo Leon</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr"/>
+          <t>Jalisco</t>
+        </is>
+      </c>
       <c r="H57" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2695,31 +2603,34 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Mystic Assembly &amp; Decorating CO</t>
+          <t>Newell Rubbermaid</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Cesar Hernandez</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>(por confirmar)</t>
+          <t>Sourcing</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>info@mysticassembly.com</t>
+          <t>cesar.hernandez@newellco.com</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Pennsylvania</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr"/>
+          <t>Baja California</t>
+        </is>
+      </c>
       <c r="H58" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2729,36 +2640,34 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Nattura Laboratorios</t>
+          <t>Pentel</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Aurora Becerra</t>
+          <t>Mauricio Perez</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Ingenieria</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>aurora.becerra@natturalabs.com</t>
+          <t>mperez@pentel.com</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Jalisco</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr"/>
+          <t>Baja California</t>
+        </is>
+      </c>
       <c r="H59" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2768,36 +2677,34 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Newell Rubbermaid</t>
+          <t>Power Sonic</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Cesar Hernandez</t>
+          <t>Ivonne Rodríguez Lesprón</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Sourcing</t>
+          <t>Jr. Manufacturing Engineer</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>cesar.hernandez@newellco.com</t>
+          <t>irodriguez@power-sonic.com</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Baja California</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr"/>
+          <t>Chihuahua</t>
+        </is>
+      </c>
       <c r="H60" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2807,36 +2714,34 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Pentel</t>
+          <t>Schwan Cosmetics (Cosmetic Colors)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Mauricio Perez</t>
+          <t>Oscar Torres</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Ingenieria</t>
+          <t>Gerente de Compra</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>mperez@pentel.com</t>
+          <t>oscar.torres@schwancosmetics.com</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Baja California</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr"/>
+          <t>Estado de Mexico</t>
+        </is>
+      </c>
       <c r="H61" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2846,36 +2751,34 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Power Sonic</t>
+          <t>Schwan Stabilo</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Ivonne Rodríguez Lesprón</t>
+          <t>Arano Lorena</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Jr. Manufacturing Engineer</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>irodriguez@power-sonic.com</t>
+          <t>lorena.arano@schwancosmetics.com</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Chihuahua</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr"/>
+          <t>DF</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2885,36 +2788,34 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Schwan Cosmetics (Cosmetic Colors)</t>
+          <t>Tae Sung Mexico</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Oscar Torres</t>
+          <t>O. Ramirez</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Gerente de Compra</t>
+          <t>Compras/Contacto</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>oscar.torres@schwancosmetics.com</t>
+          <t>oramirez@taesungmexico.com.mx</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Estado de Mexico</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr"/>
+          <t>Nuevo Leon</t>
+        </is>
+      </c>
       <c r="H63" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2924,36 +2825,34 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Schwan Stabilo</t>
+          <t>Taesung</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Arano Lorena</t>
+          <t>DIANA (DA JEONG) LEE</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Sales</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>lorena.arano@schwancosmetics.com</t>
+          <t>dianalee@taesungmexico.com.mx</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>DF</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr"/>
+          <t>Nuevo Leon</t>
+        </is>
+      </c>
       <c r="H64" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2963,36 +2862,29 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Tae Sung Mexico</t>
+          <t>Tapi America</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>O. Ramirez</t>
+          <t>Edgar Duque Duque</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Compras/Contacto</t>
+          <t>Purchasing Coordinator</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>oramirez@taesungmexico.com.mx</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>Nuevo Leon</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr"/>
+          <t>edgar.duque@gabriel.com</t>
+        </is>
+      </c>
       <c r="H65" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3002,36 +2894,34 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Taesung</t>
+          <t>Technimark</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>DIANA (DA JEONG) LEE</t>
+          <t>ADRIAN BAÑUELOS</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Sales</t>
+          <t>Manufacturing and Automation Engineer</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>dianalee@taesungmexico.com.mx</t>
+          <t>adrian.banuelos@technimark.com</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Nuevo Leon</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr"/>
+          <t>Tamaulipas</t>
+        </is>
+      </c>
       <c r="H66" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3041,31 +2931,34 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Tapi America</t>
+          <t>Tecnologías Medicas Innovadoras</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Edgar Duque Duque</t>
+          <t>Juan Antonio Hernandez</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Purchasing Coordinator</t>
+          <t>QC Manager</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>edgar.duque@gabriel.com</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr"/>
+          <t>jhernandez@tmimx.com</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Tamaulipas</t>
+        </is>
+      </c>
       <c r="H67" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3075,36 +2968,34 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Technimark</t>
+          <t>Tekmartims</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ADRIAN BAÑUELOS</t>
+          <t>Tzunalli Sifuentes Torres</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Manufacturing and Automation Engineer</t>
+          <t>Buyer</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>adrian.banuelos@technimark.com</t>
+          <t>Tzunalli.Sifuentes@tekmartims.com</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Tamaulipas</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr"/>
+          <t>Chihuahua</t>
+        </is>
+      </c>
       <c r="H68" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3114,36 +3005,34 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Tecnologías Medicas Innovadoras</t>
+          <t>Toter Inc</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Juan Antonio Hernandez</t>
+          <t>Maria Oviedo</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>QC Manager</t>
+          <t>PURCHASING ASSISTANT</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>jhernandez@tmimx.com</t>
+          <t>MOviedo@wastequip.com</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Tamaulipas</t>
-        </is>
-      </c>
-      <c r="G69" t="inlineStr"/>
+          <t>Coahuila</t>
+        </is>
+      </c>
       <c r="H69" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3153,36 +3042,34 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Tekmart Integrated Mfg</t>
+          <t>Tyden Brooks (Candados Mexicanos)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Berenice Fernandez</t>
+          <t>Patricia Garcia</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Compras MRO</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>berenice.fernandez@tekmartims.com</t>
+          <t>Patricia.Garcia@TydenBrooks.com</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Texas</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr"/>
+          <t>Nuevo Leon</t>
+        </is>
+      </c>
       <c r="H70" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3192,36 +3079,34 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Tekmartims</t>
+          <t>Unicar Plastics</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Tzunalli Sifuentes Torres</t>
+          <t>Claudia Tobón Sánchez</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Buyer</t>
+          <t>Ingeniero de Ventas</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Tzunalli.Sifuentes@tekmartims.com</t>
+          <t>ctobon@unicarmex.com</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Chihuahua</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr"/>
+          <t>Puebla</t>
+        </is>
+      </c>
       <c r="H71" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3231,36 +3116,34 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Toter Inc</t>
+          <t>Via Moda Internacional</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Maria Oviedo</t>
+          <t>E. Jaramillo</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>PURCHASING ASSISTANT</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>MOviedo@wastequip.com</t>
+          <t>ejaramillo@viamoda.com.mx</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Coahuila</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr"/>
+          <t>Jalisco</t>
+        </is>
+      </c>
       <c r="H72" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3270,36 +3153,34 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Trend Technologies</t>
+          <t>W.K.I. Automotive  México</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>O. Amezcua</t>
+          <t>Francisco  Díaz</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>Manager</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>oamezcua@trendtechnologies.com</t>
+          <t>francisco.diaz@wkiauto.com</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr"/>
+          <t>Puebla</t>
+        </is>
+      </c>
       <c r="H73" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3309,36 +3190,34 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Tyden Brooks (Candados Mexicanos)</t>
+          <t>Whirlpool</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Patricia Garcia</t>
+          <t>Ricardo Soto</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Compras MRO</t>
+          <t>Supplier Assurance Manager Procurement</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Patricia.Garcia@TydenBrooks.com</t>
+          <t>ricardo_soto@whirlpool.com</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Nuevo Leon</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr"/>
+          <t>Coahuila</t>
+        </is>
+      </c>
       <c r="H74" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3348,231 +3227,244 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Unicar Plastics</t>
+          <t>Zebra Pen</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Claudia Tobón Sánchez</t>
+          <t>Marisol Escamilla</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Ingeniero de Ventas</t>
+          <t>Planning &amp; Purchasing  Manager</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>ctobon@unicarmex.com</t>
+          <t>mescamilla@zebrapen.com</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Puebla</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr"/>
+          <t>Nuevo Leon</t>
+        </is>
+      </c>
       <c r="H75" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>B - Tier B</t>
+          <t>C - Tier C</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Via Moda Internacional</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>E. Jaramillo</t>
+          <t>(Buzon)</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>FABRICACIÓN DE PLASTISOL Y SERIGRAFÍA</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>ejaramillo@viamoda.com.mx</t>
+          <t>loya_vila@hotmail.com</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Jalisco</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr"/>
+          <t>Guanajuato</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H76" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>B - Tier B</t>
+          <t>C - Tier C</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Visteon</t>
+          <t>Baco Recolección</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>D. Sanders</t>
+          <t>(Buzon)</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Compras/Contacto</t>
+          <t>FABRICACIÓN DE RESINAS PLASTICAS</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>dsanders@visteon.com</t>
+          <t>administracion@bacorecoleccion.com</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr"/>
+          <t>Guanajuato</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H77" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>B - Tier B</t>
+          <t>C - Tier C</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>W.K.I. Automotive  México</t>
+          <t>Bulcanizados Y Moldeados De Calidad</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Francisco  Díaz</t>
+          <t>(Buzon)</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>FABRICACIÓN DE ARTÍCULOS DE PLÁSTICO</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>francisco.diaz@wkiauto.com</t>
+          <t>admonbsc@outlook.com</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Puebla</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr"/>
+          <t>Guanajuato</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H78" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>B - Tier B</t>
+          <t>C - Tier C</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Whirlpool</t>
+          <t>Conversión Termoplásticos</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Ricardo Soto</t>
+          <t>(Buzon)</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Supplier Assurance Manager Procurement</t>
+          <t>RECICLADO, MOLIENDA, TRITURADO Y TRANSFO</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>ricardo_soto@whirlpool.com</t>
+          <t>conversion.termoplasticos@gmail.com</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Coahuila</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr"/>
+          <t>Guanajuato</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H79" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>B - Tier B</t>
+          <t>C - Tier C</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Zebra Pen</t>
+          <t>Coplainsa</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Marisol Escamilla</t>
+          <t>(Buzon Logistica)</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Planning &amp; Purchasing  Manager</t>
+          <t>Logistica/Compras</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>mescamilla@zebrapen.com</t>
+          <t>logistica@coplainsa.com</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Nuevo Leon</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr"/>
+          <t>Guanajuato</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="H80" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3582,7 +3474,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Corporativo Eva</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3592,12 +3484,12 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE PLASTISOL Y SERIGRAFÍA</t>
+          <t>FABRICACIÓN DE PLASTICOS</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>loya_vila@hotmail.com</t>
+          <t>compras@productoraevadeleon.com</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3615,7 +3507,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3625,7 +3516,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Baco Recolección</t>
+          <t>Dino Stamp</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3635,12 +3526,12 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE RESINAS PLASTICAS</t>
+          <t>FABRICACIÓN DE MOLDES PARA SUELA</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>administracion@bacorecoleccion.com</t>
+          <t>gerencia@dinostamp.com.mx</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3658,7 +3549,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3668,7 +3558,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Bulcanizados Y Moldeados De Calidad</t>
+          <t>Empaques Especializados Del Centro</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3678,12 +3568,12 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE ARTÍCULOS DE PLÁSTICO</t>
+          <t>FABRICACIÓN DE INSUMOS PARA CALZADO</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>admonbsc@outlook.com</t>
+          <t>lourdesortiz@bostonplantillas.com</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3701,7 +3591,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3711,7 +3600,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Conversión Termoplásticos</t>
+          <t>Envases Universales</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3721,12 +3610,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>RECICLADO, MOLIENDA, TRITURADO Y TRANSFO</t>
+          <t>FABRICACIÓN DE ENVASES DE PLÁSTICO</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>conversion.termoplasticos@gmail.com</t>
+          <t>virginia.gonzalez@envases.mx</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3744,7 +3633,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3754,22 +3642,22 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Coplainsa</t>
+          <t>Etiquetas Rucobo</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>(Buzon Logistica)</t>
+          <t>(Buzon)</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Logistica/Compras</t>
+          <t xml:space="preserve">FABRICACIÓN DE APLICACIONES PLÁSTICAS Y </t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>logistica@coplainsa.com</t>
+          <t>rucobofacturas@yahoo.com.mx</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3787,7 +3675,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3797,7 +3684,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Corporativo Eva</t>
+          <t>Europlantas Moldeadas</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3807,12 +3694,12 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE PLASTICOS</t>
+          <t>FABRICACIÓN DE PLANTAS PARA CALZADO</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>compras@productoraevadeleon.com</t>
+          <t>europlan@grupocitrus.com</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3830,7 +3717,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3840,7 +3726,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Dino Stamp</t>
+          <t>Eva Plus Industrial</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -3850,12 +3736,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE MOLDES PARA SUELA</t>
+          <t>FABRICACIÓN DE PRODUCTOS DE PLÁSTICO</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>gerencia@dinostamp.com.mx</t>
+          <t>sandra.herrera@evaplus.com.mx</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3873,7 +3759,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3883,7 +3768,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Empaques Especializados Del Centro</t>
+          <t>Fraenkische Industrial Pipes</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3893,12 +3778,12 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE INSUMOS PARA CALZADO</t>
+          <t>FABRICACIÓN DE TUBOS Y SISTEMAS PLÁSTICO</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>lourdesortiz@bostonplantillas.com</t>
+          <t>sandra.rangel@fraenkische-mx.com</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3916,7 +3801,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3926,7 +3810,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Envases Universales</t>
+          <t>Fusion Plasticos</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3936,12 +3820,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE ENVASES DE PLÁSTICO</t>
+          <t>FABRICACIÓN DE SUELAS</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>virginia.gonzalez@envases.mx</t>
+          <t>arceliafrausto@hotmail.com</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3959,7 +3843,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3969,7 +3852,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Etiquetas Rucobo</t>
+          <t>Gomex Termoplasticos</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3979,12 +3862,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t xml:space="preserve">FABRICACIÓN DE APLICACIONES PLÁSTICAS Y </t>
+          <t>FABRICACIÓN DE TERMOPLASTICOS</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>rucobofacturas@yahoo.com.mx</t>
+          <t>talentorh@gomex.com.mx</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -4002,7 +3885,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4012,7 +3894,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Europlantas Moldeadas</t>
+          <t>Grabado Ju</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4022,12 +3904,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE PLANTAS PARA CALZADO</t>
+          <t>GRABADO Y FABRICACIÓN DE MOLDES EN GENER</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>europlan@grupocitrus.com</t>
+          <t>grabadoju@hotmail.com</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4045,7 +3927,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4055,7 +3936,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Eva Plus Industrial</t>
+          <t>Guala Dispensing Mexico S.A. De C.V.</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4065,12 +3946,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE PRODUCTOS DE PLÁSTICO</t>
+          <t>FABRICACIÓN DE ATOMIZADORES DE PLÁSTICO</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>sandra.herrera@evaplus.com.mx</t>
+          <t>veronica.solano@gualadispensing.com</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4088,7 +3969,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4098,7 +3978,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Fraenkische Industrial Pipes</t>
+          <t>Hr Proveedor</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4108,12 +3988,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE TUBOS Y SISTEMAS PLÁSTICO</t>
+          <t>COMPRAVENTA DE MATERIALES TERMOPLÁSTICOS</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>sandra.rangel@fraenkische-mx.com</t>
+          <t>hr_proveedor@hotmail.com</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -4131,7 +4011,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4141,7 +4020,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Fusion Plasticos</t>
+          <t>Imbolsa</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4151,12 +4030,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE SUELAS</t>
+          <t>FABRICACIÓN Y DISTRIBUCIÓN DE MATERIALES</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>arceliafrausto@hotmail.com</t>
+          <t>compras@gruporali.com</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4174,7 +4053,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4184,7 +4062,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Gomex Termoplasticos</t>
+          <t>Industrial Fed´S</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4194,12 +4072,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE TERMOPLASTICOS</t>
+          <t>FABRICACIÓN DE ACABADOS PARA CALZADO</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>talentorh@gomex.com.mx</t>
+          <t>jorgefernandez@feds.com.mx</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -4217,7 +4095,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4227,7 +4104,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Grabado Ju</t>
+          <t>Krah Mexico</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4237,12 +4114,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>GRABADO Y FABRICACIÓN DE MOLDES EN GENER</t>
+          <t>FABRICACIÓN DE PRODUCTOS DE PLÁSTICO</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>grabadoju@hotmail.com</t>
+          <t>a.zendejas@krahmexico.com</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -4260,7 +4137,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4270,7 +4146,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Guala Dispensing Mexico S.A. De C.V.</t>
+          <t>Macron</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4280,12 +4156,12 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE ATOMIZADORES DE PLÁSTICO</t>
+          <t xml:space="preserve">FABRICACIÓN DE PLANTILLAS Y MOLDES PARA </t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>veronica.solano@gualadispensing.com</t>
+          <t>macron-fl@hotmail.com</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -4303,7 +4179,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4313,7 +4188,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Hr Proveedor</t>
+          <t>Mecanica Stra</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -4323,12 +4198,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>COMPRAVENTA DE MATERIALES TERMOPLÁSTICOS</t>
+          <t>MOLDES Y PIEZAS ESPECIALES</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>hr_proveedor@hotmail.com</t>
+          <t>mecanicastra@hotmail.com</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -4346,7 +4221,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4356,7 +4230,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Imbolsa</t>
+          <t>Moldes Kim</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4366,12 +4240,12 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>FABRICACIÓN Y DISTRIBUCIÓN DE MATERIALES</t>
+          <t>FABRICACIÓN DE MOLDES PARA ALTA FRECUENC</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>compras@gruporali.com</t>
+          <t>claruz@live.com.mx</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -4389,7 +4263,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4399,7 +4272,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Industrial Fed´S</t>
+          <t>Moldes Sol</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4409,12 +4282,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE ACABADOS PARA CALZADO</t>
+          <t>FABRICACIÓN DE MOLDES DE ALTA FRECUENCIA</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>jorgefernandez@feds.com.mx</t>
+          <t>moldessol@yahoo.com.mx</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -4432,7 +4305,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4442,22 +4314,22 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Krah Mexico</t>
+          <t>Moriroku Technology</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>(Buzon)</t>
+          <t>(Buzon AP/Compras)</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE PRODUCTOS DE PLÁSTICO</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>a.zendejas@krahmexico.com</t>
+          <t>moriroku_ap@mtdm.mx</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -4475,7 +4347,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4485,7 +4356,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Macron</t>
+          <t>Mpe Plastics</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4495,12 +4366,12 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t xml:space="preserve">FABRICACIÓN DE PLANTILLAS Y MOLDES PARA </t>
+          <t>FABRICACIÓN DE AUTOPARTES PLÁSTICAS</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>macron-fl@hotmail.com</t>
+          <t>office.mexico@mpeplastics.com</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -4518,7 +4389,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4528,7 +4398,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Mecanica Stra</t>
+          <t>Mypi</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4538,12 +4408,12 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>MOLDES Y PIEZAS ESPECIALES</t>
+          <t>FABRICACIÓN DE MOLDES E INYECCIÓN DE PIE</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>mecanicastra@hotmail.com</t>
+          <t>adm@mypi-plasticos.com</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -4561,7 +4431,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4571,7 +4440,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Moldes Kim</t>
+          <t>Outteck</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4581,12 +4450,12 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE MOLDES PARA ALTA FRECUENC</t>
+          <t>ELABORACIÓN DE ACABADOS Y PINTURAS</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>claruz@live.com.mx</t>
+          <t>jalvarez@gruposolder.com.mx</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -4604,7 +4473,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4614,7 +4482,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Moldes Sol</t>
+          <t>Peletizados Del Rio</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4624,12 +4492,12 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE MOLDES DE ALTA FRECUENCIA</t>
+          <t>FABRICACIÓN CON ARTÍCULOS DE PLÁSTICO</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>moldessol@yahoo.com.mx</t>
+          <t>peletizadosdelrio@prodigy.net.mx</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -4647,7 +4515,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4657,22 +4524,22 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Moriroku Technology</t>
+          <t>Perfiles Y Cercos De Plástico</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>(Buzon AP/Compras)</t>
+          <t>(Buzon)</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Compras</t>
+          <t>FABRICACIÓN DE PERFILES Y CERCOS DE PLÁS</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>moriroku_ap@mtdm.mx</t>
+          <t>perfilesycercos@hotmail.com</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -4690,7 +4557,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4700,7 +4566,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Mpe Plastics</t>
+          <t>Peyga Suelas</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -4710,12 +4576,12 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE AUTOPARTES PLÁSTICAS</t>
+          <t xml:space="preserve">FABRICACIÓN DE SUELA DE TERMOPLÁSTICO Y </t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>office.mexico@mpeplastics.com</t>
+          <t>administracion@grupopeyga.com.mx</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -4733,7 +4599,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4743,7 +4608,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Mypi</t>
+          <t>Plasticos La Fiera</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -4753,12 +4618,12 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE MOLDES E INYECCIÓN DE PIE</t>
+          <t>FABRICACIÓN DE PLÁSTICOS</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>adm@mypi-plasticos.com</t>
+          <t>contabilidad@plasticoslafiera.com</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -4776,7 +4641,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4786,7 +4650,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Outteck</t>
+          <t>Plasticos Vanelli</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -4796,12 +4660,12 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>ELABORACIÓN DE ACABADOS Y PINTURAS</t>
+          <t>FABRICACIÓN DE CUBETAS DE PLÁSTICO</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>jalvarez@gruposolder.com.mx</t>
+          <t>consuelo@vanelli.com.mx</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -4819,7 +4683,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4829,7 +4692,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Peletizados Del Rio</t>
+          <t>Polimeros Y Derivados</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -4839,12 +4702,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>FABRICACIÓN CON ARTÍCULOS DE PLÁSTICO</t>
+          <t xml:space="preserve">FABRICACIÓN DE MATERIALES CELULÓSICOS Y </t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>peletizadosdelrio@prodigy.net.mx</t>
+          <t>jbriseno@polimeros.com</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -4862,7 +4725,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -4872,7 +4734,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Perfiles Y Cercos De Plástico</t>
+          <t>Polymat</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4882,12 +4744,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE PERFILES Y CERCOS DE PLÁS</t>
+          <t>FABRICACIÓN DE RESINAS PLÁSTICAS</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>perfilesycercos@hotmail.com</t>
+          <t>vtasleon@polymat.com.mx</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -4905,7 +4767,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -4915,7 +4776,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Peyga Suelas</t>
+          <t>Predemex</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -4925,12 +4786,12 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t xml:space="preserve">FABRICACIÓN DE SUELA DE TERMOPLÁSTICO Y </t>
+          <t>FABRICACIÓN DE MATERIALES PLÁSTICOS PARA</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>administracion@grupopeyga.com.mx</t>
+          <t>contraloria.predemex@gmail.com</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -4948,7 +4809,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4958,7 +4818,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Plasticos La Fiera</t>
+          <t>Provakem</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -4968,12 +4828,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE PLÁSTICOS</t>
+          <t>FABRICACIÓN DE ACABADOS PARA LA PIEL</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>contabilidad@plasticoslafiera.com</t>
+          <t>provakem22@telmex.com</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -4991,7 +4851,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5001,7 +4860,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Plasticos Vanelli</t>
+          <t>R&amp;K Chemicals</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -5011,12 +4870,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE CUBETAS DE PLÁSTICO</t>
+          <t>FABRICACIÓN DE PINTURAS PARA SUELA Y SER</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>consuelo@vanelli.com.mx</t>
+          <t>rk_chemicails@hotmail.com</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -5034,7 +4893,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5044,7 +4902,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Polimeros Y Derivados</t>
+          <t>Sandalindas</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -5054,12 +4912,12 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t xml:space="preserve">FABRICACIÓN DE MATERIALES CELULÓSICOS Y </t>
+          <t>FABRICACIÓN DE CALZADO DE PLÁSTICO</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>jbriseno@polimeros.com</t>
+          <t>sandalindascfdi@hotmail.com</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -5077,7 +4935,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5087,7 +4944,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Polymat</t>
+          <t>Simil Cuero Plymouth</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -5097,12 +4954,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE RESINAS PLÁSTICAS</t>
+          <t>VENTA DE TELAS PLÁSTICAS</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>vtasleon@polymat.com.mx</t>
+          <t>nbarajas@similcuero.com.mx</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -5120,7 +4977,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5130,7 +4986,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Predemex</t>
+          <t>Sovere De Mexico</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -5140,12 +4996,12 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE MATERIALES PLÁSTICOS PARA</t>
+          <t>FABRICACIÓN DE PRODUCTOS DE PLÁSTICO</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>contraloria.predemex@gmail.com</t>
+          <t>jorgealmaguer@sovere.com.mx</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -5163,7 +5019,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -5173,7 +5028,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Provakem</t>
+          <t>Suelas Aplasa</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -5183,12 +5038,12 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE ACABADOS PARA LA PIEL</t>
+          <t>FABRICACIÓN E INYECCIÓN DE SUELA Y PLÁST</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>provakem22@telmex.com</t>
+          <t>recursoshumanos@suelasaplasa.com</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -5206,7 +5061,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -5216,7 +5070,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>R&amp;K Chemicals</t>
+          <t>Suelas Guiver</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5226,12 +5080,12 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE PINTURAS PARA SUELA Y SER</t>
+          <t>FABRICACIÓN DE SUELAS DE TR Y MOLDES PAR</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>rk_chemicails@hotmail.com</t>
+          <t>facturassuelasguivers@hotmail.com</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -5249,7 +5103,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -5259,7 +5112,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Sandalindas</t>
+          <t>Temaplax</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -5269,12 +5122,12 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE CALZADO DE PLÁSTICO</t>
+          <t>INYECCIÓN DE PLASTICO</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>sandalindascfdi@hotmail.com</t>
+          <t>c.solis@temaplax.com</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -5292,7 +5145,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -5302,32 +5154,27 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Simil Cuero Plymouth</t>
+          <t>ABS Plastica</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>(Buzon)</t>
+          <t>(Buzon Compras)</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>VENTA DE TELAS PLÁSTICAS</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>nbarajas@similcuero.com.mx</t>
+          <t>compras@absplastica.com</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>Guanajuato</t>
-        </is>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>Sí</t>
+          <t>Puebla</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -5335,7 +5182,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -5345,32 +5191,27 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Sovere De Mexico</t>
+          <t>Industrial Corona de Mexico</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>(Buzon)</t>
+          <t>(Buzon Compras)</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE PRODUCTOS DE PLÁSTICO</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>jorgealmaguer@sovere.com.mx</t>
+          <t>compras.icm@gmail.com</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>Guanajuato</t>
-        </is>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>Sí</t>
+          <t>CDMX</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -5378,7 +5219,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -5388,32 +5228,27 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Suelas Aplasa</t>
+          <t>Moldeo de Plasticos FAR</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>(Buzon)</t>
+          <t>(Buzon Materiales)</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>FABRICACIÓN E INYECCIÓN DE SUELA Y PLÁST</t>
+          <t>Materiales / Compras</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>recursoshumanos@suelasaplasa.com</t>
+          <t>materialesFAR@ggibsa.com</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>Guanajuato</t>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>Sí</t>
+          <t>Estado de Mexico</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -5421,7 +5256,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5431,32 +5265,27 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Suelas Guiver</t>
+          <t>Productos Petigon</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>(Buzon)</t>
+          <t>(Buzon Compras)</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>FABRICACIÓN DE SUELAS DE TR Y MOLDES PAR</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>facturassuelasguivers@hotmail.com</t>
+          <t>compras@petigon.com</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>Guanajuato</t>
-        </is>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>Sí</t>
+          <t>CDMX</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -5464,7 +5293,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -5474,7 +5302,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Temaplax</t>
+          <t>Proveedores de Compuestos</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -5484,22 +5312,17 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>INYECCIÓN DE PLASTICO</t>
+          <t>Compras</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>c.solis@temaplax.com</t>
+          <t>proveecom@gmail.com</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>Guanajuato</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>Sí</t>
+          <t>CDMX</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -5507,7 +5330,6 @@
           <t>MX</t>
         </is>
       </c>
-      <c r="I125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -5517,7 +5339,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>ABS Plastica</t>
+          <t>Tecniplast</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -5532,216 +5354,19 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>compras@absplastica.com</t>
+          <t>compras@tecniplast.com.mx</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>Puebla</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr"/>
+          <t>CDMX</t>
+        </is>
+      </c>
       <c r="H126" t="inlineStr">
         <is>
           <t>MX</t>
         </is>
       </c>
-      <c r="I126" t="inlineStr"/>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>C - Tier C</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>Industrial Corona de Mexico</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>(Buzon Compras)</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>Compras</t>
-        </is>
-      </c>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>compras.icm@gmail.com</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>CDMX</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr"/>
-      <c r="H127" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="I127" t="inlineStr"/>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>C - Tier C</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>Moldeo de Plasticos FAR</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>(Buzon Materiales)</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>Materiales / Compras</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>materialesFAR@ggibsa.com</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>Estado de Mexico</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr"/>
-      <c r="H128" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="I128" t="inlineStr"/>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>C - Tier C</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>Productos Petigon</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>(Buzon Compras)</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>Compras</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>compras@petigon.com</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>CDMX</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr"/>
-      <c r="H129" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="I129" t="inlineStr"/>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>C - Tier C</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>Proveedores de Compuestos</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>(Buzon)</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>Compras</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>proveecom@gmail.com</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>CDMX</t>
-        </is>
-      </c>
-      <c r="G130" t="inlineStr"/>
-      <c r="H130" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="I130" t="inlineStr"/>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>C - Tier C</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>Tecniplast</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>(Buzon Compras)</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>Compras</t>
-        </is>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>compras@tecniplast.com.mx</t>
-        </is>
-      </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>CDMX</t>
-        </is>
-      </c>
-      <c r="G131" t="inlineStr"/>
-      <c r="H131" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="I131" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>